<commit_message>
Modif screen REG_ID read OK, autres read NOK
</commit_message>
<xml_diff>
--- a/doc/Doc_KSA/2418_DemonstrateurGraphique_Journal_KSA.xlsx
+++ b/doc/Doc_KSA/2418_DemonstrateurGraphique_Journal_KSA.xlsx
@@ -8,24 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\microchip\harmony\v2_06\apps\PROJ\PRJ_2418_demosntrateurGraphique-\doc\Doc_KSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879B47DA-C82E-4CA9-B393-EAC64BAE3911}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EDC5C17-5E94-4324-B080-8B04DC727038}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4890" yWindow="2865" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Prise en main projet =&gt; PMP</t>
   </si>
@@ -61,6 +69,9 @@
   </si>
   <si>
     <t>Modification de la lib. pour le F812</t>
+  </si>
+  <si>
+    <t>Validation lécture REG_ID / Test autre lécture NOK</t>
   </si>
 </sst>
 </file>
@@ -395,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D3:E13"/>
+  <dimension ref="D3:E14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="2"/>
@@ -492,6 +503,14 @@
         <v>11</v>
       </c>
     </row>
+    <row r="14" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D14" s="1">
+        <v>46148</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Maj. journal de travail
</commit_message>
<xml_diff>
--- a/doc/Doc_KSA/2418_DemonstrateurGraphique_Journal_KSA.xlsx
+++ b/doc/Doc_KSA/2418_DemonstrateurGraphique_Journal_KSA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\microchip\harmony\v2_06\apps\PROJ\PRJ_2418_demosntrateurGraphique-\doc\Doc_KSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EDC5C17-5E94-4324-B080-8B04DC727038}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FD123D-8CB1-483C-855B-3173C48B5752}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4890" yWindow="2865" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Prise en main projet =&gt; PMP</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>Validation lécture REG_ID / Test autre lécture NOK</t>
+  </si>
+  <si>
+    <t>Validation lécture de la ROM | Lécture RAM NOK probléme init FT812</t>
+  </si>
+  <si>
+    <t>Modif. README ajout schéma | Test corr. Init pour lire RAM</t>
   </si>
 </sst>
 </file>
@@ -406,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D3:E14"/>
+  <dimension ref="D3:E16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="2"/>
@@ -511,6 +517,22 @@
         <v>12</v>
       </c>
     </row>
+    <row r="15" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D15" s="1">
+        <v>46155</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D16" s="1">
+        <v>46162</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>